<commit_message>
Adding BVA for Product and Cart, Adding Postman collection
</commit_message>
<xml_diff>
--- a/Docs/QA-Testing/Test_Case_BVA.xlsx
+++ b/Docs/QA-Testing/Test_Case_BVA.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10821"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\task1sp4\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/admin/Downloads/Online-Store/Docs/QA-Testing/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42BD5F9A-2A01-4B3B-A514-F925A1FDAD06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFDB9E3C-D97F-7248-90BE-1A02603A5989}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1920" yWindow="7980" windowWidth="23260" windowHeight="12460" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="00_Doc_Cong_Thuc" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="549" uniqueCount="244">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="822" uniqueCount="328">
   <si>
     <t>HƯỚNG DẪN ÁP DỤNG STANDARD BOUNDARY VALUE ANALYSIS (BVA)</t>
   </si>
@@ -758,13 +758,265 @@
   </si>
   <si>
     <t>SCRUM-68</t>
+  </si>
+  <si>
+    <t>VARIABLE</t>
+  </si>
+  <si>
+    <t>BOUNDARY</t>
+  </si>
+  <si>
+    <t>VALUE</t>
+  </si>
+  <si>
+    <t>TYPE</t>
+  </si>
+  <si>
+    <t>EXPECTED</t>
+  </si>
+  <si>
+    <t>API ENDPOINT</t>
+  </si>
+  <si>
+    <t>P1-01</t>
+  </si>
+  <si>
+    <t>P1-02</t>
+  </si>
+  <si>
+    <t>P1-03</t>
+  </si>
+  <si>
+    <t>P1-04</t>
+  </si>
+  <si>
+    <t>P2-01</t>
+  </si>
+  <si>
+    <t>P2-02</t>
+  </si>
+  <si>
+    <t>P2-03</t>
+  </si>
+  <si>
+    <t>P2-04</t>
+  </si>
+  <si>
+    <t>P3-01</t>
+  </si>
+  <si>
+    <t>P3-02</t>
+  </si>
+  <si>
+    <t>P3-03</t>
+  </si>
+  <si>
+    <t>P3-04</t>
+  </si>
+  <si>
+    <t>P4-01</t>
+  </si>
+  <si>
+    <t>P4-02</t>
+  </si>
+  <si>
+    <t>P4-03</t>
+  </si>
+  <si>
+    <t>P4-04</t>
+  </si>
+  <si>
+    <t>P5-01</t>
+  </si>
+  <si>
+    <t>P5-02</t>
+  </si>
+  <si>
+    <t>P5-03</t>
+  </si>
+  <si>
+    <t>P5-04</t>
+  </si>
+  <si>
+    <t>productName</t>
+  </si>
+  <si>
+    <t>productDescription</t>
+  </si>
+  <si>
+    <t>min-1</t>
+  </si>
+  <si>
+    <t>max+1</t>
+  </si>
+  <si>
+    <t>""</t>
+  </si>
+  <si>
+    <t>"AB"</t>
+  </si>
+  <si>
+    <t>"ABC"</t>
+  </si>
+  <si>
+    <t>"A" for 30 times</t>
+  </si>
+  <si>
+    <t>"A" for 31 times</t>
+  </si>
+  <si>
+    <t>2 chars</t>
+  </si>
+  <si>
+    <t>3 chars</t>
+  </si>
+  <si>
+    <t>30 chars</t>
+  </si>
+  <si>
+    <t>31 chars</t>
+  </si>
+  <si>
+    <t>Invalid</t>
+  </si>
+  <si>
+    <t>POST /seller/product/new</t>
+  </si>
+  <si>
+    <t>min-2</t>
+  </si>
+  <si>
+    <t>max+2</t>
+  </si>
+  <si>
+    <t>"A" for 100 times</t>
+  </si>
+  <si>
+    <t>100 chars</t>
+  </si>
+  <si>
+    <t>"A" for 130 times</t>
+  </si>
+  <si>
+    <t>130 chars</t>
+  </si>
+  <si>
+    <t>Valid</t>
+  </si>
+  <si>
+    <t>Boundary</t>
+  </si>
+  <si>
+    <t>null</t>
+  </si>
+  <si>
+    <t>"D" for 201 times</t>
+  </si>
+  <si>
+    <t>"D" for 199 times</t>
+  </si>
+  <si>
+    <t>P6-NOM</t>
+  </si>
+  <si>
+    <t>ALL (P1-P5)</t>
+  </si>
+  <si>
+    <t>nominal</t>
+  </si>
+  <si>
+    <t>All valid value</t>
+  </si>
+  <si>
+    <t>Nominal</t>
+  </si>
+  <si>
+    <t>P3-NOM</t>
+  </si>
+  <si>
+    <t>ALL (C1-C2)</t>
+  </si>
+  <si>
+    <t>C1-01</t>
+  </si>
+  <si>
+    <t>C1-02</t>
+  </si>
+  <si>
+    <t>C1-03</t>
+  </si>
+  <si>
+    <t>C1-04</t>
+  </si>
+  <si>
+    <t>C2-01</t>
+  </si>
+  <si>
+    <t>C2-02</t>
+  </si>
+  <si>
+    <t>C2-03</t>
+  </si>
+  <si>
+    <t>C2-04</t>
+  </si>
+  <si>
+    <t>productId="D002", quantity=1</t>
+  </si>
+  <si>
+    <t>STD</t>
+  </si>
+  <si>
+    <t>Robustness</t>
+  </si>
+  <si>
+    <t>R-P01</t>
+  </si>
+  <si>
+    <t>R-P02</t>
+  </si>
+  <si>
+    <t>R-P03</t>
+  </si>
+  <si>
+    <t>R-P04</t>
+  </si>
+  <si>
+    <t>R-P05</t>
+  </si>
+  <si>
+    <t>R-P06</t>
+  </si>
+  <si>
+    <t>R-P07</t>
+  </si>
+  <si>
+    <t>below min</t>
+  </si>
+  <si>
+    <t>"A" for 32 times</t>
+  </si>
+  <si>
+    <t>"A" for 102 times</t>
+  </si>
+  <si>
+    <t>"A' for 201 times</t>
+  </si>
+  <si>
+    <t>32 chars</t>
+  </si>
+  <si>
+    <t>102 chars</t>
+  </si>
+  <si>
+    <t>201 chars</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="14" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -829,8 +1081,31 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="10">
+  <fills count="16">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -881,6 +1156,42 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="3">
     <border>
@@ -924,7 +1235,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="57">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -976,16 +1287,6 @@
     <xf numFmtId="0" fontId="9" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -998,6 +1299,72 @@
     <xf numFmtId="0" fontId="10" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="11" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="11" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="12" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="12" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="12" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="13" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1306,7 +1673,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G27"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
     <col min="2" max="2" width="55" customWidth="1"/>
@@ -1316,29 +1683,29 @@
     <col min="6" max="6" width="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="22" t="s">
+    <row r="1" spans="1:7" ht="25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="26" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
-      <c r="E1" s="20"/>
-      <c r="F1" s="20"/>
-      <c r="G1" s="20"/>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A3" s="21" t="s">
+      <c r="B1" s="24"/>
+      <c r="C1" s="24"/>
+      <c r="D1" s="24"/>
+      <c r="E1" s="24"/>
+      <c r="F1" s="24"/>
+      <c r="G1" s="24"/>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A3" s="27" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="20"/>
-      <c r="C3" s="20"/>
-      <c r="D3" s="20"/>
-      <c r="E3" s="20"/>
-      <c r="F3" s="20"/>
-      <c r="G3" s="20"/>
-    </row>
-    <row r="4" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B3" s="24"/>
+      <c r="C3" s="24"/>
+      <c r="D3" s="24"/>
+      <c r="E3" s="24"/>
+      <c r="F3" s="24"/>
+      <c r="G3" s="24"/>
+    </row>
+    <row r="4" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>2</v>
       </c>
@@ -1346,7 +1713,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -1354,7 +1721,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>6</v>
       </c>
@@ -1362,18 +1729,18 @@
         <v>7</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A8" s="21" t="s">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A8" s="27" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="20"/>
-      <c r="C8" s="20"/>
-      <c r="D8" s="20"/>
-      <c r="E8" s="20"/>
-      <c r="F8" s="20"/>
-      <c r="G8" s="20"/>
-    </row>
-    <row r="9" spans="1:7" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="B8" s="24"/>
+      <c r="C8" s="24"/>
+      <c r="D8" s="24"/>
+      <c r="E8" s="24"/>
+      <c r="F8" s="24"/>
+      <c r="G8" s="24"/>
+    </row>
+    <row r="9" spans="1:7" ht="17" x14ac:dyDescent="0.2">
       <c r="A9" s="3" t="s">
         <v>9</v>
       </c>
@@ -1393,7 +1760,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" s="4" t="s">
         <v>15</v>
       </c>
@@ -1413,7 +1780,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="11" spans="1:7" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" ht="28" x14ac:dyDescent="0.2">
       <c r="A11" s="5" t="s">
         <v>19</v>
       </c>
@@ -1433,7 +1800,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" s="4" t="s">
         <v>23</v>
       </c>
@@ -1453,18 +1820,18 @@
         <v>26</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A14" s="21" t="s">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A14" s="27" t="s">
         <v>27</v>
       </c>
-      <c r="B14" s="20"/>
-      <c r="C14" s="20"/>
-      <c r="D14" s="20"/>
-      <c r="E14" s="20"/>
-      <c r="F14" s="20"/>
-      <c r="G14" s="20"/>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B14" s="24"/>
+      <c r="C14" s="24"/>
+      <c r="D14" s="24"/>
+      <c r="E14" s="24"/>
+      <c r="F14" s="24"/>
+      <c r="G14" s="24"/>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>28</v>
       </c>
@@ -1472,7 +1839,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>30</v>
       </c>
@@ -1480,18 +1847,18 @@
         <v>31</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A18" s="21" t="s">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A18" s="27" t="s">
         <v>32</v>
       </c>
-      <c r="B18" s="20"/>
-      <c r="C18" s="20"/>
-      <c r="D18" s="20"/>
-      <c r="E18" s="20"/>
-      <c r="F18" s="20"/>
-      <c r="G18" s="20"/>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B18" s="24"/>
+      <c r="C18" s="24"/>
+      <c r="D18" s="24"/>
+      <c r="E18" s="24"/>
+      <c r="F18" s="24"/>
+      <c r="G18" s="24"/>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>33</v>
       </c>
@@ -1499,7 +1866,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>35</v>
       </c>
@@ -1507,80 +1874,80 @@
         <v>36</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A22" s="21" t="s">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A22" s="27" t="s">
         <v>37</v>
       </c>
-      <c r="B22" s="20"/>
-      <c r="C22" s="20"/>
-      <c r="D22" s="20"/>
-      <c r="E22" s="20"/>
-      <c r="F22" s="20"/>
-      <c r="G22" s="20"/>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A23" s="19" t="s">
+      <c r="B22" s="24"/>
+      <c r="C22" s="24"/>
+      <c r="D22" s="24"/>
+      <c r="E22" s="24"/>
+      <c r="F22" s="24"/>
+      <c r="G22" s="24"/>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A23" s="28" t="s">
         <v>38</v>
       </c>
-      <c r="B23" s="20"/>
-      <c r="C23" s="20"/>
-      <c r="D23" s="20"/>
-      <c r="E23" s="20"/>
-      <c r="F23" s="20"/>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A24" s="19" t="s">
+      <c r="B23" s="24"/>
+      <c r="C23" s="24"/>
+      <c r="D23" s="24"/>
+      <c r="E23" s="24"/>
+      <c r="F23" s="24"/>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A24" s="28" t="s">
         <v>39</v>
       </c>
-      <c r="B24" s="20"/>
-      <c r="C24" s="20"/>
-      <c r="D24" s="20"/>
-      <c r="E24" s="20"/>
-      <c r="F24" s="20"/>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A25" s="19" t="s">
+      <c r="B24" s="24"/>
+      <c r="C24" s="24"/>
+      <c r="D24" s="24"/>
+      <c r="E24" s="24"/>
+      <c r="F24" s="24"/>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A25" s="28" t="s">
         <v>40</v>
       </c>
-      <c r="B25" s="20"/>
-      <c r="C25" s="20"/>
-      <c r="D25" s="20"/>
-      <c r="E25" s="20"/>
-      <c r="F25" s="20"/>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A26" s="19" t="s">
+      <c r="B25" s="24"/>
+      <c r="C25" s="24"/>
+      <c r="D25" s="24"/>
+      <c r="E25" s="24"/>
+      <c r="F25" s="24"/>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A26" s="28" t="s">
         <v>41</v>
       </c>
-      <c r="B26" s="20"/>
-      <c r="C26" s="20"/>
-      <c r="D26" s="20"/>
-      <c r="E26" s="20"/>
-      <c r="F26" s="20"/>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A27" s="19" t="s">
+      <c r="B26" s="24"/>
+      <c r="C26" s="24"/>
+      <c r="D26" s="24"/>
+      <c r="E26" s="24"/>
+      <c r="F26" s="24"/>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A27" s="28" t="s">
         <v>42</v>
       </c>
-      <c r="B27" s="20"/>
-      <c r="C27" s="20"/>
-      <c r="D27" s="20"/>
-      <c r="E27" s="20"/>
-      <c r="F27" s="20"/>
+      <c r="B27" s="24"/>
+      <c r="C27" s="24"/>
+      <c r="D27" s="24"/>
+      <c r="E27" s="24"/>
+      <c r="F27" s="24"/>
     </row>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A18:G18"/>
-    <mergeCell ref="A8:G8"/>
-    <mergeCell ref="A3:G3"/>
-    <mergeCell ref="A22:G22"/>
     <mergeCell ref="A27:F27"/>
     <mergeCell ref="A26:F26"/>
     <mergeCell ref="A25:F25"/>
     <mergeCell ref="A24:F24"/>
     <mergeCell ref="A14:G14"/>
     <mergeCell ref="A23:F23"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A18:G18"/>
+    <mergeCell ref="A8:G8"/>
+    <mergeCell ref="A3:G3"/>
+    <mergeCell ref="A22:G22"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1589,7 +1956,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:H16"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
@@ -1597,36 +1964,36 @@
     <col min="4" max="8" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A1" s="24" t="s">
+    <row r="1" spans="1:8" ht="18" x14ac:dyDescent="0.2">
+      <c r="A1" s="25" t="s">
         <v>43</v>
       </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
-      <c r="E1" s="20"/>
-      <c r="F1" s="20"/>
-      <c r="G1" s="20"/>
-      <c r="H1" s="20"/>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="B1" s="24"/>
+      <c r="C1" s="24"/>
+      <c r="D1" s="24"/>
+      <c r="E1" s="24"/>
+      <c r="F1" s="24"/>
+      <c r="G1" s="24"/>
+      <c r="H1" s="24"/>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A4" s="23" t="s">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A4" s="29" t="s">
         <v>203</v>
       </c>
-      <c r="B4" s="20"/>
-      <c r="C4" s="20"/>
-      <c r="D4" s="20"/>
-      <c r="E4" s="20"/>
-      <c r="F4" s="20"/>
-      <c r="G4" s="20"/>
-      <c r="H4" s="20"/>
-    </row>
-    <row r="6" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B4" s="24"/>
+      <c r="C4" s="24"/>
+      <c r="D4" s="24"/>
+      <c r="E4" s="24"/>
+      <c r="F4" s="24"/>
+      <c r="G4" s="24"/>
+      <c r="H4" s="24"/>
+    </row>
+    <row r="6" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A6" s="3" t="s">
         <v>45</v>
       </c>
@@ -1652,7 +2019,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" s="5" t="s">
         <v>53</v>
       </c>
@@ -1678,7 +2045,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A8" s="4" t="s">
         <v>61</v>
       </c>
@@ -1704,7 +2071,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" s="5" t="s">
         <v>67</v>
       </c>
@@ -1730,7 +2097,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A10" s="4" t="s">
         <v>73</v>
       </c>
@@ -1756,7 +2123,7 @@
         <v>207</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A11" s="5" t="s">
         <v>76</v>
       </c>
@@ -1782,22 +2149,22 @@
         <v>82</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>86</v>
       </c>
@@ -1814,7 +2181,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:M36"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="18.6640625" customWidth="1"/>
     <col min="2" max="2" width="22" customWidth="1"/>
@@ -1830,39 +2197,39 @@
     <col min="13" max="13" width="11.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A1" s="24" t="s">
+    <row r="1" spans="1:13" ht="18" x14ac:dyDescent="0.2">
+      <c r="A1" s="25" t="s">
         <v>87</v>
       </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
-      <c r="E1" s="20"/>
-      <c r="F1" s="20"/>
-      <c r="G1" s="20"/>
-      <c r="H1" s="20"/>
-      <c r="I1" s="20"/>
-      <c r="J1" s="20"/>
-      <c r="K1" s="20"/>
-      <c r="L1" s="20"/>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A3" s="25" t="s">
+      <c r="B1" s="24"/>
+      <c r="C1" s="24"/>
+      <c r="D1" s="24"/>
+      <c r="E1" s="24"/>
+      <c r="F1" s="24"/>
+      <c r="G1" s="24"/>
+      <c r="H1" s="24"/>
+      <c r="I1" s="24"/>
+      <c r="J1" s="24"/>
+      <c r="K1" s="24"/>
+      <c r="L1" s="24"/>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A3" s="23" t="s">
         <v>88</v>
       </c>
-      <c r="B3" s="20"/>
-      <c r="C3" s="20"/>
-      <c r="D3" s="20"/>
-      <c r="E3" s="20"/>
-      <c r="F3" s="20"/>
-      <c r="G3" s="20"/>
-      <c r="H3" s="20"/>
-      <c r="I3" s="20"/>
-      <c r="J3" s="20"/>
-      <c r="K3" s="20"/>
-      <c r="L3" s="20"/>
-    </row>
-    <row r="5" spans="1:13" s="28" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B3" s="24"/>
+      <c r="C3" s="24"/>
+      <c r="D3" s="24"/>
+      <c r="E3" s="24"/>
+      <c r="F3" s="24"/>
+      <c r="G3" s="24"/>
+      <c r="H3" s="24"/>
+      <c r="I3" s="24"/>
+      <c r="J3" s="24"/>
+      <c r="K3" s="24"/>
+      <c r="L3" s="24"/>
+    </row>
+    <row r="5" spans="1:13" s="20" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A5" s="7" t="s">
         <v>89</v>
       </c>
@@ -1903,7 +2270,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="6" spans="1:13" s="28" customFormat="1" ht="30" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:13" s="20" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A6" s="8" t="s">
         <v>96</v>
       </c>
@@ -1938,9 +2305,9 @@
         <v>233</v>
       </c>
       <c r="L6" s="8"/>
-      <c r="M6" s="30"/>
-    </row>
-    <row r="7" spans="1:13" s="28" customFormat="1" ht="30" x14ac:dyDescent="0.3">
+      <c r="M6" s="22"/>
+    </row>
+    <row r="7" spans="1:13" s="20" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A7" s="10" t="s">
         <v>103</v>
       </c>
@@ -1977,9 +2344,9 @@
       <c r="L7" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="M7" s="29"/>
-    </row>
-    <row r="8" spans="1:13" s="28" customFormat="1" ht="30" x14ac:dyDescent="0.3">
+      <c r="M7" s="21"/>
+    </row>
+    <row r="8" spans="1:13" s="20" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A8" s="12" t="s">
         <v>105</v>
       </c>
@@ -2016,9 +2383,9 @@
       <c r="L8" s="12" t="s">
         <v>57</v>
       </c>
-      <c r="M8" s="30"/>
-    </row>
-    <row r="9" spans="1:13" s="28" customFormat="1" ht="60" x14ac:dyDescent="0.3">
+      <c r="M8" s="22"/>
+    </row>
+    <row r="9" spans="1:13" s="20" customFormat="1" ht="68" x14ac:dyDescent="0.2">
       <c r="A9" s="10" t="s">
         <v>107</v>
       </c>
@@ -2055,9 +2422,9 @@
       <c r="L9" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="M9" s="29"/>
-    </row>
-    <row r="10" spans="1:13" s="28" customFormat="1" ht="60" x14ac:dyDescent="0.3">
+      <c r="M9" s="21"/>
+    </row>
+    <row r="10" spans="1:13" s="20" customFormat="1" ht="68" x14ac:dyDescent="0.2">
       <c r="A10" s="12" t="s">
         <v>108</v>
       </c>
@@ -2094,9 +2461,9 @@
       <c r="L10" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="M10" s="30"/>
-    </row>
-    <row r="11" spans="1:13" s="28" customFormat="1" ht="30" x14ac:dyDescent="0.3">
+      <c r="M10" s="22"/>
+    </row>
+    <row r="11" spans="1:13" s="20" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A11" s="10" t="s">
         <v>109</v>
       </c>
@@ -2133,9 +2500,9 @@
       <c r="L11" s="10" t="s">
         <v>64</v>
       </c>
-      <c r="M11" s="29"/>
-    </row>
-    <row r="12" spans="1:13" s="28" customFormat="1" ht="30" x14ac:dyDescent="0.3">
+      <c r="M11" s="21"/>
+    </row>
+    <row r="12" spans="1:13" s="20" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A12" s="12" t="s">
         <v>111</v>
       </c>
@@ -2172,9 +2539,9 @@
       <c r="L12" s="12" t="s">
         <v>65</v>
       </c>
-      <c r="M12" s="30"/>
-    </row>
-    <row r="13" spans="1:13" s="28" customFormat="1" ht="75" x14ac:dyDescent="0.3">
+      <c r="M12" s="22"/>
+    </row>
+    <row r="13" spans="1:13" s="20" customFormat="1" ht="85" x14ac:dyDescent="0.2">
       <c r="A13" s="10" t="s">
         <v>113</v>
       </c>
@@ -2211,9 +2578,9 @@
       <c r="L13" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="M13" s="29"/>
-    </row>
-    <row r="14" spans="1:13" s="28" customFormat="1" ht="75" x14ac:dyDescent="0.3">
+      <c r="M13" s="21"/>
+    </row>
+    <row r="14" spans="1:13" s="20" customFormat="1" ht="85" x14ac:dyDescent="0.2">
       <c r="A14" s="12" t="s">
         <v>114</v>
       </c>
@@ -2250,9 +2617,9 @@
       <c r="L14" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="M14" s="30"/>
-    </row>
-    <row r="15" spans="1:13" s="28" customFormat="1" ht="30" x14ac:dyDescent="0.3">
+      <c r="M14" s="22"/>
+    </row>
+    <row r="15" spans="1:13" s="20" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A15" s="10" t="s">
         <v>115</v>
       </c>
@@ -2289,9 +2656,9 @@
       <c r="L15" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="M15" s="29"/>
-    </row>
-    <row r="16" spans="1:13" s="28" customFormat="1" ht="30" x14ac:dyDescent="0.3">
+      <c r="M15" s="21"/>
+    </row>
+    <row r="16" spans="1:13" s="20" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A16" s="12" t="s">
         <v>117</v>
       </c>
@@ -2328,9 +2695,9 @@
       <c r="L16" s="12" t="s">
         <v>70</v>
       </c>
-      <c r="M16" s="30"/>
-    </row>
-    <row r="17" spans="1:13" s="28" customFormat="1" ht="30" x14ac:dyDescent="0.3">
+      <c r="M16" s="22"/>
+    </row>
+    <row r="17" spans="1:13" s="20" customFormat="1" ht="34" x14ac:dyDescent="0.2">
       <c r="A17" s="10" t="s">
         <v>119</v>
       </c>
@@ -2367,9 +2734,9 @@
       <c r="L17" s="10" t="s">
         <v>72</v>
       </c>
-      <c r="M17" s="29"/>
-    </row>
-    <row r="18" spans="1:13" s="28" customFormat="1" ht="30" x14ac:dyDescent="0.3">
+      <c r="M17" s="21"/>
+    </row>
+    <row r="18" spans="1:13" s="20" customFormat="1" ht="34" x14ac:dyDescent="0.2">
       <c r="A18" s="12" t="s">
         <v>120</v>
       </c>
@@ -2406,9 +2773,9 @@
       <c r="L18" s="12" t="s">
         <v>58</v>
       </c>
-      <c r="M18" s="30"/>
-    </row>
-    <row r="19" spans="1:13" s="28" customFormat="1" ht="30" x14ac:dyDescent="0.3">
+      <c r="M18" s="22"/>
+    </row>
+    <row r="19" spans="1:13" s="20" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A19" s="10" t="s">
         <v>121</v>
       </c>
@@ -2445,9 +2812,9 @@
       <c r="L19" s="10" t="s">
         <v>206</v>
       </c>
-      <c r="M19" s="29"/>
-    </row>
-    <row r="20" spans="1:13" s="28" customFormat="1" ht="30" x14ac:dyDescent="0.3">
+      <c r="M19" s="21"/>
+    </row>
+    <row r="20" spans="1:13" s="20" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A20" s="12" t="s">
         <v>122</v>
       </c>
@@ -2484,9 +2851,9 @@
       <c r="L20" s="12" t="s">
         <v>208</v>
       </c>
-      <c r="M20" s="30"/>
-    </row>
-    <row r="21" spans="1:13" s="28" customFormat="1" ht="30" x14ac:dyDescent="0.3">
+      <c r="M20" s="22"/>
+    </row>
+    <row r="21" spans="1:13" s="20" customFormat="1" ht="34" x14ac:dyDescent="0.2">
       <c r="A21" s="10" t="s">
         <v>124</v>
       </c>
@@ -2523,9 +2890,9 @@
       <c r="L21" s="10" t="s">
         <v>75</v>
       </c>
-      <c r="M21" s="29"/>
-    </row>
-    <row r="22" spans="1:13" s="28" customFormat="1" ht="30" x14ac:dyDescent="0.3">
+      <c r="M21" s="21"/>
+    </row>
+    <row r="22" spans="1:13" s="20" customFormat="1" ht="34" x14ac:dyDescent="0.2">
       <c r="A22" s="12" t="s">
         <v>125</v>
       </c>
@@ -2562,9 +2929,9 @@
       <c r="L22" s="12" t="s">
         <v>207</v>
       </c>
-      <c r="M22" s="30"/>
-    </row>
-    <row r="23" spans="1:13" s="28" customFormat="1" ht="15" x14ac:dyDescent="0.3">
+      <c r="M22" s="22"/>
+    </row>
+    <row r="23" spans="1:13" s="20" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A23" s="10" t="s">
         <v>126</v>
       </c>
@@ -2601,9 +2968,9 @@
       <c r="L23" s="10" t="s">
         <v>79</v>
       </c>
-      <c r="M23" s="29"/>
-    </row>
-    <row r="24" spans="1:13" s="28" customFormat="1" ht="15" x14ac:dyDescent="0.3">
+      <c r="M23" s="21"/>
+    </row>
+    <row r="24" spans="1:13" s="20" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A24" s="12" t="s">
         <v>128</v>
       </c>
@@ -2640,9 +3007,9 @@
       <c r="L24" s="12" t="s">
         <v>56</v>
       </c>
-      <c r="M24" s="30"/>
-    </row>
-    <row r="25" spans="1:13" s="28" customFormat="1" ht="120" x14ac:dyDescent="0.3">
+      <c r="M24" s="22"/>
+    </row>
+    <row r="25" spans="1:13" s="20" customFormat="1" ht="119" x14ac:dyDescent="0.2">
       <c r="A25" s="10" t="s">
         <v>130</v>
       </c>
@@ -2679,9 +3046,9 @@
       <c r="L25" s="10" t="s">
         <v>81</v>
       </c>
-      <c r="M25" s="29"/>
-    </row>
-    <row r="26" spans="1:13" s="28" customFormat="1" ht="120" x14ac:dyDescent="0.3">
+      <c r="M25" s="21"/>
+    </row>
+    <row r="26" spans="1:13" s="20" customFormat="1" ht="119" x14ac:dyDescent="0.2">
       <c r="A26" s="12" t="s">
         <v>131</v>
       </c>
@@ -2718,9 +3085,9 @@
       <c r="L26" s="12" t="s">
         <v>82</v>
       </c>
-      <c r="M26" s="30"/>
-    </row>
-    <row r="27" spans="1:13" s="28" customFormat="1" ht="30" x14ac:dyDescent="0.3">
+      <c r="M26" s="22"/>
+    </row>
+    <row r="27" spans="1:13" s="20" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A27" s="13" t="s">
         <v>220</v>
       </c>
@@ -2739,7 +3106,7 @@
       <c r="F27" s="13" t="s">
         <v>226</v>
       </c>
-      <c r="G27" s="27" t="s">
+      <c r="G27" s="19" t="s">
         <v>101</v>
       </c>
       <c r="H27" s="13" t="s">
@@ -2757,11 +3124,11 @@
       <c r="L27" s="13" t="s">
         <v>64</v>
       </c>
-      <c r="M27" s="29" t="s">
+      <c r="M27" s="21" t="s">
         <v>240</v>
       </c>
     </row>
-    <row r="28" spans="1:13" s="28" customFormat="1" ht="30" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:13" s="20" customFormat="1" ht="34" x14ac:dyDescent="0.2">
       <c r="A28" s="14" t="s">
         <v>221</v>
       </c>
@@ -2780,7 +3147,7 @@
       <c r="F28" s="14" t="s">
         <v>228</v>
       </c>
-      <c r="G28" s="27" t="s">
+      <c r="G28" s="19" t="s">
         <v>235</v>
       </c>
       <c r="H28" s="14" t="s">
@@ -2798,11 +3165,11 @@
       <c r="L28" s="14" t="s">
         <v>229</v>
       </c>
-      <c r="M28" s="30" t="s">
+      <c r="M28" s="22" t="s">
         <v>241</v>
       </c>
     </row>
-    <row r="29" spans="1:13" s="28" customFormat="1" ht="30" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:13" s="20" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A29" s="13" t="s">
         <v>222</v>
       </c>
@@ -2821,7 +3188,7 @@
       <c r="F29" s="13" t="s">
         <v>100</v>
       </c>
-      <c r="G29" s="27" t="s">
+      <c r="G29" s="19" t="s">
         <v>236</v>
       </c>
       <c r="H29" s="13" t="s">
@@ -2839,11 +3206,11 @@
       <c r="L29" s="13" t="s">
         <v>79</v>
       </c>
-      <c r="M29" s="29" t="s">
+      <c r="M29" s="21" t="s">
         <v>242</v>
       </c>
     </row>
-    <row r="30" spans="1:13" s="28" customFormat="1" ht="60" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:13" s="20" customFormat="1" ht="68" x14ac:dyDescent="0.2">
       <c r="A30" s="14" t="s">
         <v>223</v>
       </c>
@@ -2862,7 +3229,7 @@
       <c r="F30" s="14" t="s">
         <v>100</v>
       </c>
-      <c r="G30" s="27" t="s">
+      <c r="G30" s="19" t="s">
         <v>237</v>
       </c>
       <c r="H30" s="14" t="s">
@@ -2880,31 +3247,31 @@
       <c r="L30" s="14" t="s">
         <v>232</v>
       </c>
-      <c r="M30" s="30" t="s">
+      <c r="M30" s="22" t="s">
         <v>243</v>
       </c>
     </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A32" s="1" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>238</v>
       </c>
@@ -2925,45 +3292,47 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:H11"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:H44"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
     <col min="3" max="3" width="26" customWidth="1"/>
-    <col min="4" max="8" width="18" customWidth="1"/>
+    <col min="4" max="6" width="18" customWidth="1"/>
+    <col min="7" max="7" width="29.6640625" customWidth="1"/>
+    <col min="8" max="8" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A1" s="24" t="s">
+    <row r="1" spans="1:8" ht="18" x14ac:dyDescent="0.2">
+      <c r="A1" s="25" t="s">
         <v>136</v>
       </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
-      <c r="E1" s="20"/>
-      <c r="F1" s="20"/>
-      <c r="G1" s="20"/>
-      <c r="H1" s="20"/>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="B1" s="24"/>
+      <c r="C1" s="24"/>
+      <c r="D1" s="24"/>
+      <c r="E1" s="24"/>
+      <c r="F1" s="24"/>
+      <c r="G1" s="24"/>
+      <c r="H1" s="24"/>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A4" s="26" t="s">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A4" s="30" t="s">
         <v>137</v>
       </c>
-      <c r="B4" s="20"/>
-      <c r="C4" s="20"/>
-      <c r="D4" s="20"/>
-      <c r="E4" s="20"/>
-      <c r="F4" s="20"/>
-      <c r="G4" s="20"/>
-      <c r="H4" s="20"/>
-    </row>
-    <row r="6" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B4" s="24"/>
+      <c r="C4" s="24"/>
+      <c r="D4" s="24"/>
+      <c r="E4" s="24"/>
+      <c r="F4" s="24"/>
+      <c r="G4" s="24"/>
+      <c r="H4" s="24"/>
+    </row>
+    <row r="6" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A6" s="3" t="s">
         <v>45</v>
       </c>
@@ -2989,7 +3358,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" s="4" t="s">
         <v>138</v>
       </c>
@@ -3015,7 +3384,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A8" s="4" t="s">
         <v>146</v>
       </c>
@@ -3041,22 +3410,717 @@
         <v>153</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A11" s="20" t="s">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A11" s="24" t="s">
         <v>155</v>
       </c>
-      <c r="B11" s="20"/>
-      <c r="C11" s="20"/>
-      <c r="D11" s="20"/>
-      <c r="E11" s="20"/>
-      <c r="F11" s="20"/>
-      <c r="G11" s="20"/>
-      <c r="H11" s="20"/>
+      <c r="B11" s="24"/>
+      <c r="C11" s="24"/>
+      <c r="D11" s="24"/>
+      <c r="E11" s="24"/>
+      <c r="F11" s="24"/>
+      <c r="G11" s="24"/>
+      <c r="H11" s="24"/>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A13" s="32" t="s">
+        <v>89</v>
+      </c>
+      <c r="B13" s="32" t="s">
+        <v>244</v>
+      </c>
+      <c r="C13" s="32" t="s">
+        <v>245</v>
+      </c>
+      <c r="D13" s="32" t="s">
+        <v>246</v>
+      </c>
+      <c r="E13" s="32" t="s">
+        <v>247</v>
+      </c>
+      <c r="F13" s="32" t="s">
+        <v>248</v>
+      </c>
+      <c r="G13" s="32" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A14" s="34" t="s">
+        <v>250</v>
+      </c>
+      <c r="B14" s="35" t="s">
+        <v>188</v>
+      </c>
+      <c r="C14" s="34" t="s">
+        <v>272</v>
+      </c>
+      <c r="D14" s="34" t="s">
+        <v>275</v>
+      </c>
+      <c r="E14" s="34" t="s">
+        <v>279</v>
+      </c>
+      <c r="F14" s="34">
+        <v>400</v>
+      </c>
+      <c r="G14" s="36" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A15" s="34" t="s">
+        <v>251</v>
+      </c>
+      <c r="B15" s="35" t="s">
+        <v>188</v>
+      </c>
+      <c r="C15" s="34" t="s">
+        <v>48</v>
+      </c>
+      <c r="D15" s="34" t="s">
+        <v>276</v>
+      </c>
+      <c r="E15" s="34" t="s">
+        <v>280</v>
+      </c>
+      <c r="F15" s="34">
+        <v>200</v>
+      </c>
+      <c r="G15" s="36" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A16" s="34" t="s">
+        <v>252</v>
+      </c>
+      <c r="B16" s="35" t="s">
+        <v>188</v>
+      </c>
+      <c r="C16" s="34" t="s">
+        <v>52</v>
+      </c>
+      <c r="D16" s="34" t="s">
+        <v>277</v>
+      </c>
+      <c r="E16" s="34" t="s">
+        <v>281</v>
+      </c>
+      <c r="F16" s="34">
+        <v>200</v>
+      </c>
+      <c r="G16" s="37" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A17" s="34" t="s">
+        <v>253</v>
+      </c>
+      <c r="B17" s="35" t="s">
+        <v>188</v>
+      </c>
+      <c r="C17" s="34" t="s">
+        <v>273</v>
+      </c>
+      <c r="D17" s="34" t="s">
+        <v>278</v>
+      </c>
+      <c r="E17" s="34" t="s">
+        <v>282</v>
+      </c>
+      <c r="F17" s="34">
+        <v>400</v>
+      </c>
+      <c r="G17" s="37" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A18" s="38" t="s">
+        <v>254</v>
+      </c>
+      <c r="B18" s="39" t="s">
+        <v>270</v>
+      </c>
+      <c r="C18" s="38" t="s">
+        <v>272</v>
+      </c>
+      <c r="D18" s="38" t="s">
+        <v>275</v>
+      </c>
+      <c r="E18" s="38" t="s">
+        <v>279</v>
+      </c>
+      <c r="F18" s="38">
+        <v>400</v>
+      </c>
+      <c r="G18" s="40" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A19" s="38" t="s">
+        <v>255</v>
+      </c>
+      <c r="B19" s="39" t="s">
+        <v>270</v>
+      </c>
+      <c r="C19" s="38" t="s">
+        <v>48</v>
+      </c>
+      <c r="D19" s="38" t="s">
+        <v>276</v>
+      </c>
+      <c r="E19" s="38" t="s">
+        <v>280</v>
+      </c>
+      <c r="F19" s="38">
+        <v>200</v>
+      </c>
+      <c r="G19" s="40" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A20" s="38" t="s">
+        <v>256</v>
+      </c>
+      <c r="B20" s="39" t="s">
+        <v>270</v>
+      </c>
+      <c r="C20" s="38" t="s">
+        <v>52</v>
+      </c>
+      <c r="D20" s="38" t="s">
+        <v>287</v>
+      </c>
+      <c r="E20" s="38" t="s">
+        <v>288</v>
+      </c>
+      <c r="F20" s="38">
+        <v>200</v>
+      </c>
+      <c r="G20" s="41" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A21" s="38" t="s">
+        <v>257</v>
+      </c>
+      <c r="B21" s="39" t="s">
+        <v>270</v>
+      </c>
+      <c r="C21" s="38" t="s">
+        <v>273</v>
+      </c>
+      <c r="D21" s="38" t="s">
+        <v>289</v>
+      </c>
+      <c r="E21" s="38" t="s">
+        <v>290</v>
+      </c>
+      <c r="F21" s="38">
+        <v>400</v>
+      </c>
+      <c r="G21" s="41" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A22" s="53" t="s">
+        <v>258</v>
+      </c>
+      <c r="B22" s="54" t="s">
+        <v>138</v>
+      </c>
+      <c r="C22" s="53" t="s">
+        <v>272</v>
+      </c>
+      <c r="D22" s="53">
+        <v>0</v>
+      </c>
+      <c r="E22" s="53" t="s">
+        <v>283</v>
+      </c>
+      <c r="F22" s="53">
+        <v>400</v>
+      </c>
+      <c r="G22" s="55" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A23" s="53" t="s">
+        <v>259</v>
+      </c>
+      <c r="B23" s="54" t="s">
+        <v>138</v>
+      </c>
+      <c r="C23" s="53" t="s">
+        <v>48</v>
+      </c>
+      <c r="D23" s="53" t="s">
+        <v>141</v>
+      </c>
+      <c r="E23" s="53" t="s">
+        <v>292</v>
+      </c>
+      <c r="F23" s="53">
+        <v>200</v>
+      </c>
+      <c r="G23" s="56" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A24" s="53" t="s">
+        <v>260</v>
+      </c>
+      <c r="B24" s="54" t="s">
+        <v>138</v>
+      </c>
+      <c r="C24" s="53" t="s">
+        <v>52</v>
+      </c>
+      <c r="D24" s="53">
+        <v>999999</v>
+      </c>
+      <c r="E24" s="53" t="s">
+        <v>292</v>
+      </c>
+      <c r="F24" s="53">
+        <v>200</v>
+      </c>
+      <c r="G24" s="56" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A25" s="53" t="s">
+        <v>261</v>
+      </c>
+      <c r="B25" s="54" t="s">
+        <v>138</v>
+      </c>
+      <c r="C25" s="53" t="s">
+        <v>273</v>
+      </c>
+      <c r="D25" s="53">
+        <v>1000000</v>
+      </c>
+      <c r="E25" s="53" t="s">
+        <v>291</v>
+      </c>
+      <c r="F25" s="53">
+        <v>200</v>
+      </c>
+      <c r="G25" s="55" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A26" s="49" t="s">
+        <v>262</v>
+      </c>
+      <c r="B26" s="50" t="s">
+        <v>146</v>
+      </c>
+      <c r="C26" s="49" t="s">
+        <v>272</v>
+      </c>
+      <c r="D26" s="49">
+        <v>-1</v>
+      </c>
+      <c r="E26" s="49" t="s">
+        <v>283</v>
+      </c>
+      <c r="F26" s="49">
+        <v>400</v>
+      </c>
+      <c r="G26" s="51" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A27" s="49" t="s">
+        <v>263</v>
+      </c>
+      <c r="B27" s="50" t="s">
+        <v>146</v>
+      </c>
+      <c r="C27" s="49" t="s">
+        <v>48</v>
+      </c>
+      <c r="D27" s="49">
+        <v>0</v>
+      </c>
+      <c r="E27" s="49" t="s">
+        <v>292</v>
+      </c>
+      <c r="F27" s="49">
+        <v>200</v>
+      </c>
+      <c r="G27" s="51" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A28" s="49" t="s">
+        <v>264</v>
+      </c>
+      <c r="B28" s="50" t="s">
+        <v>146</v>
+      </c>
+      <c r="C28" s="49" t="s">
+        <v>52</v>
+      </c>
+      <c r="D28" s="49">
+        <v>999999</v>
+      </c>
+      <c r="E28" s="49" t="s">
+        <v>292</v>
+      </c>
+      <c r="F28" s="49">
+        <v>200</v>
+      </c>
+      <c r="G28" s="52" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A29" s="49" t="s">
+        <v>265</v>
+      </c>
+      <c r="B29" s="50" t="s">
+        <v>146</v>
+      </c>
+      <c r="C29" s="49" t="s">
+        <v>273</v>
+      </c>
+      <c r="D29" s="49">
+        <v>1000000</v>
+      </c>
+      <c r="E29" s="49" t="s">
+        <v>291</v>
+      </c>
+      <c r="F29" s="49">
+        <v>200</v>
+      </c>
+      <c r="G29" s="51" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A30" s="42" t="s">
+        <v>266</v>
+      </c>
+      <c r="B30" s="43" t="s">
+        <v>271</v>
+      </c>
+      <c r="C30" s="42" t="s">
+        <v>272</v>
+      </c>
+      <c r="D30" s="42" t="s">
+        <v>293</v>
+      </c>
+      <c r="E30" s="42" t="s">
+        <v>292</v>
+      </c>
+      <c r="F30" s="42">
+        <v>200</v>
+      </c>
+      <c r="G30" s="44" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A31" s="42" t="s">
+        <v>267</v>
+      </c>
+      <c r="B31" s="43" t="s">
+        <v>271</v>
+      </c>
+      <c r="C31" s="42" t="s">
+        <v>48</v>
+      </c>
+      <c r="D31" s="42" t="s">
+        <v>274</v>
+      </c>
+      <c r="E31" s="42" t="s">
+        <v>292</v>
+      </c>
+      <c r="F31" s="42">
+        <v>200</v>
+      </c>
+      <c r="G31" s="44" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A32" s="42" t="s">
+        <v>268</v>
+      </c>
+      <c r="B32" s="43" t="s">
+        <v>271</v>
+      </c>
+      <c r="C32" s="42" t="s">
+        <v>52</v>
+      </c>
+      <c r="D32" s="42" t="s">
+        <v>295</v>
+      </c>
+      <c r="E32" s="42" t="s">
+        <v>291</v>
+      </c>
+      <c r="F32" s="42">
+        <v>200</v>
+      </c>
+      <c r="G32" s="45" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A33" s="42" t="s">
+        <v>269</v>
+      </c>
+      <c r="B33" s="43" t="s">
+        <v>271</v>
+      </c>
+      <c r="C33" s="42" t="s">
+        <v>273</v>
+      </c>
+      <c r="D33" s="42" t="s">
+        <v>294</v>
+      </c>
+      <c r="E33" s="42" t="s">
+        <v>283</v>
+      </c>
+      <c r="F33" s="42">
+        <v>400</v>
+      </c>
+      <c r="G33" s="44" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A34" s="46" t="s">
+        <v>296</v>
+      </c>
+      <c r="B34" s="47" t="s">
+        <v>297</v>
+      </c>
+      <c r="C34" s="46" t="s">
+        <v>298</v>
+      </c>
+      <c r="D34" s="46" t="s">
+        <v>299</v>
+      </c>
+      <c r="E34" s="46" t="s">
+        <v>300</v>
+      </c>
+      <c r="F34" s="46">
+        <v>200</v>
+      </c>
+      <c r="G34" s="48" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A36" s="38" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A37" s="32" t="s">
+        <v>89</v>
+      </c>
+      <c r="B37" s="32" t="s">
+        <v>244</v>
+      </c>
+      <c r="C37" s="32" t="s">
+        <v>245</v>
+      </c>
+      <c r="D37" s="32" t="s">
+        <v>246</v>
+      </c>
+      <c r="E37" s="32" t="s">
+        <v>247</v>
+      </c>
+      <c r="F37" s="32" t="s">
+        <v>248</v>
+      </c>
+      <c r="G37" s="32" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A38" s="31" t="s">
+        <v>314</v>
+      </c>
+      <c r="B38" s="33" t="s">
+        <v>188</v>
+      </c>
+      <c r="C38" s="31" t="s">
+        <v>285</v>
+      </c>
+      <c r="D38" s="31" t="s">
+        <v>293</v>
+      </c>
+      <c r="E38" s="31" t="s">
+        <v>313</v>
+      </c>
+      <c r="F38" s="31">
+        <v>400</v>
+      </c>
+      <c r="G38" s="31" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A39" s="31" t="s">
+        <v>315</v>
+      </c>
+      <c r="B39" s="33" t="s">
+        <v>188</v>
+      </c>
+      <c r="C39" s="31" t="s">
+        <v>286</v>
+      </c>
+      <c r="D39" s="31" t="s">
+        <v>322</v>
+      </c>
+      <c r="E39" s="31" t="s">
+        <v>325</v>
+      </c>
+      <c r="F39" s="31">
+        <v>400</v>
+      </c>
+      <c r="G39" s="31" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A40" s="31" t="s">
+        <v>316</v>
+      </c>
+      <c r="B40" s="33" t="s">
+        <v>270</v>
+      </c>
+      <c r="C40" s="31" t="s">
+        <v>285</v>
+      </c>
+      <c r="D40" s="31" t="s">
+        <v>293</v>
+      </c>
+      <c r="E40" s="31" t="s">
+        <v>313</v>
+      </c>
+      <c r="F40" s="31">
+        <v>400</v>
+      </c>
+      <c r="G40" s="31" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A41" s="31" t="s">
+        <v>317</v>
+      </c>
+      <c r="B41" s="33" t="s">
+        <v>270</v>
+      </c>
+      <c r="C41" s="31" t="s">
+        <v>286</v>
+      </c>
+      <c r="D41" s="31" t="s">
+        <v>323</v>
+      </c>
+      <c r="E41" s="31" t="s">
+        <v>326</v>
+      </c>
+      <c r="F41" s="31">
+        <v>400</v>
+      </c>
+      <c r="G41" s="31" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A42" s="31" t="s">
+        <v>318</v>
+      </c>
+      <c r="B42" s="33" t="s">
+        <v>138</v>
+      </c>
+      <c r="C42" s="31" t="s">
+        <v>321</v>
+      </c>
+      <c r="D42" s="31">
+        <v>-1</v>
+      </c>
+      <c r="E42" s="31" t="s">
+        <v>313</v>
+      </c>
+      <c r="F42" s="31">
+        <v>400</v>
+      </c>
+      <c r="G42" s="31" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A43" s="31" t="s">
+        <v>319</v>
+      </c>
+      <c r="B43" s="33" t="s">
+        <v>146</v>
+      </c>
+      <c r="C43" s="31" t="s">
+        <v>285</v>
+      </c>
+      <c r="D43" s="31">
+        <v>-2</v>
+      </c>
+      <c r="E43" s="31" t="s">
+        <v>313</v>
+      </c>
+      <c r="F43" s="31">
+        <v>400</v>
+      </c>
+      <c r="G43" s="31" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A44" s="31" t="s">
+        <v>320</v>
+      </c>
+      <c r="B44" s="33" t="s">
+        <v>271</v>
+      </c>
+      <c r="C44" s="31" t="s">
+        <v>286</v>
+      </c>
+      <c r="D44" s="31" t="s">
+        <v>324</v>
+      </c>
+      <c r="E44" s="31" t="s">
+        <v>327</v>
+      </c>
+      <c r="F44" s="31">
+        <v>400</v>
+      </c>
+      <c r="G44" s="31" t="s">
+        <v>284</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -3064,6 +4128,7 @@
     <mergeCell ref="A11:H11"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
+  <phoneticPr fontId="7" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3071,7 +4136,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:J19"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
     <col min="2" max="2" width="22" customWidth="1"/>
@@ -3084,35 +4149,35 @@
     <col min="10" max="10" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A1" s="24" t="s">
+    <row r="1" spans="1:10" ht="18" x14ac:dyDescent="0.2">
+      <c r="A1" s="25" t="s">
         <v>156</v>
       </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
-      <c r="E1" s="20"/>
-      <c r="F1" s="20"/>
-      <c r="G1" s="20"/>
-      <c r="H1" s="20"/>
-      <c r="I1" s="20"/>
-      <c r="J1" s="20"/>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A3" s="25" t="s">
+      <c r="B1" s="24"/>
+      <c r="C1" s="24"/>
+      <c r="D1" s="24"/>
+      <c r="E1" s="24"/>
+      <c r="F1" s="24"/>
+      <c r="G1" s="24"/>
+      <c r="H1" s="24"/>
+      <c r="I1" s="24"/>
+      <c r="J1" s="24"/>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A3" s="23" t="s">
         <v>157</v>
       </c>
-      <c r="B3" s="20"/>
-      <c r="C3" s="20"/>
-      <c r="D3" s="20"/>
-      <c r="E3" s="20"/>
-      <c r="F3" s="20"/>
-      <c r="G3" s="20"/>
-      <c r="H3" s="20"/>
-      <c r="I3" s="20"/>
-      <c r="J3" s="20"/>
-    </row>
-    <row r="5" spans="1:10" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="B3" s="24"/>
+      <c r="C3" s="24"/>
+      <c r="D3" s="24"/>
+      <c r="E3" s="24"/>
+      <c r="F3" s="24"/>
+      <c r="G3" s="24"/>
+      <c r="H3" s="24"/>
+      <c r="I3" s="24"/>
+      <c r="J3" s="24"/>
+    </row>
+    <row r="5" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="A5" s="3" t="s">
         <v>89</v>
       </c>
@@ -3144,7 +4209,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:10" ht="28" x14ac:dyDescent="0.2">
       <c r="A6" s="6" t="s">
         <v>159</v>
       </c>
@@ -3168,7 +4233,7 @@
       <c r="I6" s="6"/>
       <c r="J6" s="6"/>
     </row>
-    <row r="7" spans="1:10" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A7" s="5" t="s">
         <v>161</v>
       </c>
@@ -3194,7 +4259,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="8" spans="1:10" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A8" s="4" t="s">
         <v>164</v>
       </c>
@@ -3218,7 +4283,7 @@
       <c r="I8" s="4"/>
       <c r="J8" s="4"/>
     </row>
-    <row r="9" spans="1:10" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A9" s="5" t="s">
         <v>165</v>
       </c>
@@ -3242,7 +4307,7 @@
       <c r="I9" s="5"/>
       <c r="J9" s="5"/>
     </row>
-    <row r="10" spans="1:10" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A10" s="4" t="s">
         <v>166</v>
       </c>
@@ -3268,7 +4333,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A11" s="5" t="s">
         <v>168</v>
       </c>
@@ -3294,7 +4359,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="12" spans="1:10" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A12" s="4" t="s">
         <v>170</v>
       </c>
@@ -3318,7 +4383,7 @@
       <c r="I12" s="4"/>
       <c r="J12" s="4"/>
     </row>
-    <row r="13" spans="1:10" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A13" s="5" t="s">
         <v>171</v>
       </c>
@@ -3342,7 +4407,7 @@
       <c r="I13" s="5"/>
       <c r="J13" s="5"/>
     </row>
-    <row r="14" spans="1:10" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A14" s="4" t="s">
         <v>172</v>
       </c>
@@ -3366,22 +4431,22 @@
       <c r="I14" s="4"/>
       <c r="J14" s="4"/>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
         <v>173</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>174</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>176</v>
       </c>
@@ -3397,44 +4462,47 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:H10"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:H32"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="3" width="26" customWidth="1"/>
-    <col min="4" max="8" width="18" customWidth="1"/>
+    <col min="4" max="4" width="28.33203125" customWidth="1"/>
+    <col min="5" max="6" width="18" customWidth="1"/>
+    <col min="7" max="7" width="21.83203125" customWidth="1"/>
+    <col min="8" max="8" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A1" s="24" t="s">
+    <row r="1" spans="1:8" ht="18" x14ac:dyDescent="0.2">
+      <c r="A1" s="25" t="s">
         <v>177</v>
       </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
-      <c r="E1" s="20"/>
-      <c r="F1" s="20"/>
-      <c r="G1" s="20"/>
-      <c r="H1" s="20"/>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="B1" s="24"/>
+      <c r="C1" s="24"/>
+      <c r="D1" s="24"/>
+      <c r="E1" s="24"/>
+      <c r="F1" s="24"/>
+      <c r="G1" s="24"/>
+      <c r="H1" s="24"/>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A4" s="26" t="s">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A4" s="30" t="s">
         <v>178</v>
       </c>
-      <c r="B4" s="20"/>
-      <c r="C4" s="20"/>
-      <c r="D4" s="20"/>
-      <c r="E4" s="20"/>
-      <c r="F4" s="20"/>
-      <c r="G4" s="20"/>
-      <c r="H4" s="20"/>
-    </row>
-    <row r="6" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B4" s="24"/>
+      <c r="C4" s="24"/>
+      <c r="D4" s="24"/>
+      <c r="E4" s="24"/>
+      <c r="F4" s="24"/>
+      <c r="G4" s="24"/>
+      <c r="H4" s="24"/>
+    </row>
+    <row r="6" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A6" s="3" t="s">
         <v>45</v>
       </c>
@@ -3460,7 +4528,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" s="4" t="s">
         <v>25</v>
       </c>
@@ -3486,22 +4554,425 @@
         <v>183</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
         <v>184</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A10" s="20" t="s">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A10" s="24" t="s">
         <v>185</v>
       </c>
-      <c r="B10" s="20"/>
-      <c r="C10" s="20"/>
-      <c r="D10" s="20"/>
-      <c r="E10" s="20"/>
-      <c r="F10" s="20"/>
-      <c r="G10" s="20"/>
-      <c r="H10" s="20"/>
+      <c r="B10" s="24"/>
+      <c r="C10" s="24"/>
+      <c r="D10" s="24"/>
+      <c r="E10" s="24"/>
+      <c r="F10" s="24"/>
+      <c r="G10" s="24"/>
+      <c r="H10" s="24"/>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A12" s="38" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A13" s="32" t="s">
+        <v>89</v>
+      </c>
+      <c r="B13" s="32" t="s">
+        <v>244</v>
+      </c>
+      <c r="C13" s="32" t="s">
+        <v>245</v>
+      </c>
+      <c r="D13" s="32" t="s">
+        <v>246</v>
+      </c>
+      <c r="E13" s="32" t="s">
+        <v>247</v>
+      </c>
+      <c r="F13" s="32" t="s">
+        <v>248</v>
+      </c>
+      <c r="G13" s="32" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A14" s="34" t="s">
+        <v>303</v>
+      </c>
+      <c r="B14" s="35" t="s">
+        <v>188</v>
+      </c>
+      <c r="C14" s="34" t="s">
+        <v>272</v>
+      </c>
+      <c r="D14" s="34" t="s">
+        <v>275</v>
+      </c>
+      <c r="E14" s="34" t="s">
+        <v>279</v>
+      </c>
+      <c r="F14" s="34">
+        <v>400</v>
+      </c>
+      <c r="G14" s="36" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A15" s="34" t="s">
+        <v>304</v>
+      </c>
+      <c r="B15" s="35" t="s">
+        <v>188</v>
+      </c>
+      <c r="C15" s="34" t="s">
+        <v>48</v>
+      </c>
+      <c r="D15" s="34" t="s">
+        <v>276</v>
+      </c>
+      <c r="E15" s="34" t="s">
+        <v>280</v>
+      </c>
+      <c r="F15" s="34">
+        <v>200</v>
+      </c>
+      <c r="G15" s="36" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A16" s="34" t="s">
+        <v>305</v>
+      </c>
+      <c r="B16" s="35" t="s">
+        <v>188</v>
+      </c>
+      <c r="C16" s="34" t="s">
+        <v>52</v>
+      </c>
+      <c r="D16" s="34" t="s">
+        <v>277</v>
+      </c>
+      <c r="E16" s="34" t="s">
+        <v>281</v>
+      </c>
+      <c r="F16" s="34">
+        <v>200</v>
+      </c>
+      <c r="G16" s="36" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A17" s="34" t="s">
+        <v>306</v>
+      </c>
+      <c r="B17" s="35" t="s">
+        <v>188</v>
+      </c>
+      <c r="C17" s="34" t="s">
+        <v>273</v>
+      </c>
+      <c r="D17" s="34" t="s">
+        <v>278</v>
+      </c>
+      <c r="E17" s="34" t="s">
+        <v>282</v>
+      </c>
+      <c r="F17" s="34">
+        <v>400</v>
+      </c>
+      <c r="G17" s="36" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A18" s="38" t="s">
+        <v>307</v>
+      </c>
+      <c r="B18" s="39" t="s">
+        <v>25</v>
+      </c>
+      <c r="C18" s="38" t="s">
+        <v>272</v>
+      </c>
+      <c r="D18" s="38">
+        <v>0</v>
+      </c>
+      <c r="E18" s="38" t="s">
+        <v>283</v>
+      </c>
+      <c r="F18" s="38">
+        <v>400</v>
+      </c>
+      <c r="G18" s="40" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A19" s="38" t="s">
+        <v>308</v>
+      </c>
+      <c r="B19" s="39" t="s">
+        <v>25</v>
+      </c>
+      <c r="C19" s="38" t="s">
+        <v>48</v>
+      </c>
+      <c r="D19" s="38">
+        <v>1</v>
+      </c>
+      <c r="E19" s="38" t="s">
+        <v>292</v>
+      </c>
+      <c r="F19" s="38">
+        <v>200</v>
+      </c>
+      <c r="G19" s="40" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A20" s="38" t="s">
+        <v>309</v>
+      </c>
+      <c r="B20" s="39" t="s">
+        <v>25</v>
+      </c>
+      <c r="C20" s="38" t="s">
+        <v>52</v>
+      </c>
+      <c r="D20" s="38">
+        <v>999999</v>
+      </c>
+      <c r="E20" s="38" t="s">
+        <v>292</v>
+      </c>
+      <c r="F20" s="38">
+        <v>200</v>
+      </c>
+      <c r="G20" s="40" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A21" s="38" t="s">
+        <v>310</v>
+      </c>
+      <c r="B21" s="39" t="s">
+        <v>25</v>
+      </c>
+      <c r="C21" s="38" t="s">
+        <v>273</v>
+      </c>
+      <c r="D21" s="38">
+        <v>1000000</v>
+      </c>
+      <c r="E21" s="38" t="s">
+        <v>291</v>
+      </c>
+      <c r="F21" s="38">
+        <v>200</v>
+      </c>
+      <c r="G21" s="40" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A22" s="53" t="s">
+        <v>301</v>
+      </c>
+      <c r="B22" s="54" t="s">
+        <v>302</v>
+      </c>
+      <c r="C22" s="53" t="s">
+        <v>298</v>
+      </c>
+      <c r="D22" s="53" t="s">
+        <v>311</v>
+      </c>
+      <c r="E22" s="53" t="s">
+        <v>300</v>
+      </c>
+      <c r="F22" s="53">
+        <v>200</v>
+      </c>
+      <c r="G22" s="55" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A24" s="38" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A25" s="32" t="s">
+        <v>89</v>
+      </c>
+      <c r="B25" s="32" t="s">
+        <v>244</v>
+      </c>
+      <c r="C25" s="32" t="s">
+        <v>245</v>
+      </c>
+      <c r="D25" s="32" t="s">
+        <v>246</v>
+      </c>
+      <c r="E25" s="32" t="s">
+        <v>247</v>
+      </c>
+      <c r="F25" s="32" t="s">
+        <v>248</v>
+      </c>
+      <c r="G25" s="32" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A26" s="31" t="s">
+        <v>314</v>
+      </c>
+      <c r="B26" s="33" t="s">
+        <v>188</v>
+      </c>
+      <c r="C26" s="31" t="s">
+        <v>285</v>
+      </c>
+      <c r="D26" s="31" t="s">
+        <v>293</v>
+      </c>
+      <c r="E26" s="31" t="s">
+        <v>313</v>
+      </c>
+      <c r="F26" s="31">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A27" s="31" t="s">
+        <v>315</v>
+      </c>
+      <c r="B27" s="33" t="s">
+        <v>188</v>
+      </c>
+      <c r="C27" s="31" t="s">
+        <v>286</v>
+      </c>
+      <c r="D27" s="31" t="s">
+        <v>322</v>
+      </c>
+      <c r="E27" s="31" t="s">
+        <v>325</v>
+      </c>
+      <c r="F27" s="31">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A28" s="31" t="s">
+        <v>316</v>
+      </c>
+      <c r="B28" s="33" t="s">
+        <v>270</v>
+      </c>
+      <c r="C28" s="31" t="s">
+        <v>285</v>
+      </c>
+      <c r="D28" s="31" t="s">
+        <v>293</v>
+      </c>
+      <c r="E28" s="31" t="s">
+        <v>313</v>
+      </c>
+      <c r="F28" s="31">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A29" s="31" t="s">
+        <v>317</v>
+      </c>
+      <c r="B29" s="33" t="s">
+        <v>270</v>
+      </c>
+      <c r="C29" s="31" t="s">
+        <v>286</v>
+      </c>
+      <c r="D29" s="31" t="s">
+        <v>323</v>
+      </c>
+      <c r="E29" s="31" t="s">
+        <v>326</v>
+      </c>
+      <c r="F29" s="31">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A30" s="31" t="s">
+        <v>318</v>
+      </c>
+      <c r="B30" s="33" t="s">
+        <v>138</v>
+      </c>
+      <c r="C30" s="31" t="s">
+        <v>321</v>
+      </c>
+      <c r="D30" s="31">
+        <v>-1</v>
+      </c>
+      <c r="E30" s="31" t="s">
+        <v>313</v>
+      </c>
+      <c r="F30" s="31">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A31" s="31" t="s">
+        <v>319</v>
+      </c>
+      <c r="B31" s="33" t="s">
+        <v>146</v>
+      </c>
+      <c r="C31" s="31" t="s">
+        <v>285</v>
+      </c>
+      <c r="D31" s="31">
+        <v>-2</v>
+      </c>
+      <c r="E31" s="31" t="s">
+        <v>313</v>
+      </c>
+      <c r="F31" s="31">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A32" s="31" t="s">
+        <v>320</v>
+      </c>
+      <c r="B32" s="33" t="s">
+        <v>271</v>
+      </c>
+      <c r="C32" s="31" t="s">
+        <v>286</v>
+      </c>
+      <c r="D32" s="31" t="s">
+        <v>324</v>
+      </c>
+      <c r="E32" s="31" t="s">
+        <v>327</v>
+      </c>
+      <c r="F32" s="31">
+        <v>400</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -3509,6 +4980,7 @@
     <mergeCell ref="A10:H10"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
+  <phoneticPr fontId="7" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3516,7 +4988,7 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:J15"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
     <col min="2" max="2" width="20" customWidth="1"/>
@@ -3528,35 +5000,35 @@
     <col min="10" max="10" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A1" s="24" t="s">
+    <row r="1" spans="1:10" ht="18" x14ac:dyDescent="0.2">
+      <c r="A1" s="25" t="s">
         <v>186</v>
       </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
-      <c r="E1" s="20"/>
-      <c r="F1" s="20"/>
-      <c r="G1" s="20"/>
-      <c r="H1" s="20"/>
-      <c r="I1" s="20"/>
-      <c r="J1" s="20"/>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A3" s="25" t="s">
+      <c r="B1" s="24"/>
+      <c r="C1" s="24"/>
+      <c r="D1" s="24"/>
+      <c r="E1" s="24"/>
+      <c r="F1" s="24"/>
+      <c r="G1" s="24"/>
+      <c r="H1" s="24"/>
+      <c r="I1" s="24"/>
+      <c r="J1" s="24"/>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A3" s="23" t="s">
         <v>187</v>
       </c>
-      <c r="B3" s="20"/>
-      <c r="C3" s="20"/>
-      <c r="D3" s="20"/>
-      <c r="E3" s="20"/>
-      <c r="F3" s="20"/>
-      <c r="G3" s="20"/>
-      <c r="H3" s="20"/>
-      <c r="I3" s="20"/>
-      <c r="J3" s="20"/>
-    </row>
-    <row r="5" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B3" s="24"/>
+      <c r="C3" s="24"/>
+      <c r="D3" s="24"/>
+      <c r="E3" s="24"/>
+      <c r="F3" s="24"/>
+      <c r="G3" s="24"/>
+      <c r="H3" s="24"/>
+      <c r="I3" s="24"/>
+      <c r="J3" s="24"/>
+    </row>
+    <row r="5" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="A5" s="3" t="s">
         <v>89</v>
       </c>
@@ -3588,7 +5060,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:10" ht="28" x14ac:dyDescent="0.2">
       <c r="A6" s="6" t="s">
         <v>190</v>
       </c>
@@ -3614,7 +5086,7 @@
       </c>
       <c r="J6" s="6"/>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A7" s="5" t="s">
         <v>195</v>
       </c>
@@ -3642,7 +5114,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A8" s="4" t="s">
         <v>197</v>
       </c>
@@ -3668,7 +5140,7 @@
       </c>
       <c r="J8" s="4"/>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A9" s="5" t="s">
         <v>198</v>
       </c>
@@ -3694,7 +5166,7 @@
       </c>
       <c r="J9" s="5"/>
     </row>
-    <row r="10" spans="1:10" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:10" ht="28" x14ac:dyDescent="0.2">
       <c r="A10" s="4" t="s">
         <v>199</v>
       </c>
@@ -3722,22 +5194,22 @@
         <v>167</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>200</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>201</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>202</v>
       </c>

</xml_diff>